<commit_message>
Add hero block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (10):
- MIGRATION.md
- blocks/hero/hero.css
- styles/styles.css
- tools/importer/backups/general/import-general-v1.bundle.js
- tools/importer/backups/general/import-general-v1.js
- tools/importer/backups/general/manifest.md
- tools/importer/import-general-v1.bundle.js
- tools/importer/import-general-v1.js
- tools/importer/reports/en/home/who-we-are.report.json
- tools/importer/reports/import-general-v1.report.xlsx
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-general-v1.report.xlsx
+++ b/tools/importer/reports/import-general-v1.report.xlsx
@@ -73,7 +73,7 @@
     <t>en/home/who-we-are.report.json</t>
   </si>
   <si>
-    <t>["hero-text-up","default-content(intro)","columns(history,image-right)","section-metadata(yellow-intro)","columns(evert,image-left)","section-metadata(yellow-columns)","default-content(supporters)","cards-tiles"]</t>
+    <t>["hero-text-up","default-content(intro)","columns(history,image-right)","columns(evert,image-left)","section-metadata(yellow-band)","default-content(supporters)","cards-tiles","spacer(trailing-black-band)"]</t>
   </si>
   <si>
     <t>en/home/who-we-are</t>
@@ -82,7 +82,7 @@
     <t>general</t>
   </si>
   <si>
-    <t>2026-09-08T07:38:30.023Z</t>
+    <t>2026-09-08T08:34:00.217Z</t>
   </si>
   <si>
     <t>Who We Are</t>

</xml_diff>